<commit_message>
Auto commit 09-07-2026 17:28:48.60
</commit_message>
<xml_diff>
--- a/Side Bar Files/GWD Data/PAMR39.xlsx
+++ b/Side Bar Files/GWD Data/PAMR39.xlsx
@@ -10653,7 +10653,7 @@
   <numFmts count="1">
     <numFmt numFmtId="177" formatCode="dd-mm-yyyy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -10667,14 +10667,8 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Cambria"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
-      <sz val="9"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Cambria"/>
       <family val="2"/>
@@ -10722,18 +10716,15 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -11174,7 +11165,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C24C9A95-C2E8-4752-B54F-EE16ED21BAA6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03728CD3-0ED3-43DD-B1B5-57361B31BAA6}">
   <dimension ref="A1:J1741"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <sheetData>
@@ -12977,7 +12968,7 @@
       <c r="B57" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C57" s="4" t="s">
+      <c r="C57" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D57" s="2" t="s">
@@ -13297,7 +13288,7 @@
       <c r="B67" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C67" s="4" t="s">
+      <c r="C67" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D67" s="2" t="s">
@@ -13937,7 +13928,7 @@
       <c r="B87" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C87" s="4" t="s">
+      <c r="C87" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D87" s="2" t="s">
@@ -14705,7 +14696,7 @@
       <c r="B111" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C111" s="4" t="s">
+      <c r="C111" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D111" s="2" t="s">
@@ -15569,7 +15560,7 @@
       <c r="B138" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C138" s="4" t="s">
+      <c r="C138" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D138" s="2" t="s">
@@ -16369,7 +16360,7 @@
       <c r="B163" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C163" s="4" t="s">
+      <c r="C163" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D163" s="2" t="s">
@@ -17137,7 +17128,7 @@
       <c r="B187" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C187" s="5"/>
+      <c r="C187" s="4"/>
       <c r="D187" s="2" t="s">
         <v>393</v>
       </c>
@@ -17167,7 +17158,7 @@
       <c r="B188" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C188" s="5"/>
+      <c r="C188" s="4"/>
       <c r="D188" s="2" t="s">
         <v>395</v>
       </c>
@@ -17197,7 +17188,7 @@
       <c r="B189" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C189" s="5"/>
+      <c r="C189" s="4"/>
       <c r="D189" s="2" t="s">
         <v>397</v>
       </c>
@@ -17227,7 +17218,7 @@
       <c r="B190" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C190" s="5"/>
+      <c r="C190" s="4"/>
       <c r="D190" s="2" t="s">
         <v>399</v>
       </c>
@@ -17257,7 +17248,7 @@
       <c r="B191" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C191" s="5"/>
+      <c r="C191" s="4"/>
       <c r="D191" s="2" t="s">
         <v>401</v>
       </c>
@@ -17287,7 +17278,7 @@
       <c r="B192" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C192" s="5"/>
+      <c r="C192" s="4"/>
       <c r="D192" s="2" t="s">
         <v>403</v>
       </c>
@@ -17317,7 +17308,7 @@
       <c r="B193" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C193" s="5"/>
+      <c r="C193" s="4"/>
       <c r="D193" s="2" t="s">
         <v>405</v>
       </c>
@@ -17347,7 +17338,7 @@
       <c r="B194" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C194" s="5"/>
+      <c r="C194" s="4"/>
       <c r="D194" s="2" t="s">
         <v>407</v>
       </c>
@@ -17377,7 +17368,7 @@
       <c r="B195" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C195" s="5"/>
+      <c r="C195" s="4"/>
       <c r="D195" s="2" t="s">
         <v>409</v>
       </c>
@@ -17407,7 +17398,7 @@
       <c r="B196" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C196" s="5"/>
+      <c r="C196" s="4"/>
       <c r="D196" s="2" t="s">
         <v>411</v>
       </c>
@@ -17437,7 +17428,7 @@
       <c r="B197" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C197" s="5"/>
+      <c r="C197" s="4"/>
       <c r="D197" s="2" t="s">
         <v>413</v>
       </c>
@@ -17467,7 +17458,7 @@
       <c r="B198" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C198" s="5"/>
+      <c r="C198" s="4"/>
       <c r="D198" s="2" t="s">
         <v>415</v>
       </c>
@@ -17497,7 +17488,7 @@
       <c r="B199" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C199" s="5"/>
+      <c r="C199" s="4"/>
       <c r="D199" s="2" t="s">
         <v>417</v>
       </c>
@@ -17527,7 +17518,7 @@
       <c r="B200" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C200" s="5"/>
+      <c r="C200" s="4"/>
       <c r="D200" s="2" t="s">
         <v>419</v>
       </c>
@@ -17557,7 +17548,7 @@
       <c r="B201" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C201" s="5"/>
+      <c r="C201" s="4"/>
       <c r="D201" s="2" t="s">
         <v>421</v>
       </c>
@@ -17587,7 +17578,7 @@
       <c r="B202" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C202" s="5"/>
+      <c r="C202" s="4"/>
       <c r="D202" s="2" t="s">
         <v>423</v>
       </c>
@@ -17617,7 +17608,7 @@
       <c r="B203" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C203" s="5"/>
+      <c r="C203" s="4"/>
       <c r="D203" s="2" t="s">
         <v>425</v>
       </c>
@@ -17647,7 +17638,7 @@
       <c r="B204" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C204" s="5"/>
+      <c r="C204" s="4"/>
       <c r="D204" s="2" t="s">
         <v>427</v>
       </c>
@@ -17677,7 +17668,7 @@
       <c r="B205" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C205" s="5"/>
+      <c r="C205" s="4"/>
       <c r="D205" s="2" t="s">
         <v>429</v>
       </c>
@@ -17707,7 +17698,7 @@
       <c r="B206" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C206" s="5"/>
+      <c r="C206" s="4"/>
       <c r="D206" s="2" t="s">
         <v>431</v>
       </c>
@@ -17737,7 +17728,7 @@
       <c r="B207" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C207" s="5"/>
+      <c r="C207" s="4"/>
       <c r="D207" s="2" t="s">
         <v>433</v>
       </c>
@@ -17767,7 +17758,7 @@
       <c r="B208" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C208" s="5"/>
+      <c r="C208" s="4"/>
       <c r="D208" s="2" t="s">
         <v>435</v>
       </c>
@@ -17797,7 +17788,7 @@
       <c r="B209" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C209" s="5"/>
+      <c r="C209" s="4"/>
       <c r="D209" s="2" t="s">
         <v>437</v>
       </c>
@@ -17827,7 +17818,7 @@
       <c r="B210" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C210" s="5"/>
+      <c r="C210" s="4"/>
       <c r="D210" s="2" t="s">
         <v>439</v>
       </c>
@@ -17857,7 +17848,7 @@
       <c r="B211" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C211" s="5"/>
+      <c r="C211" s="4"/>
       <c r="D211" s="2" t="s">
         <v>441</v>
       </c>
@@ -17887,7 +17878,7 @@
       <c r="B212" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C212" s="5"/>
+      <c r="C212" s="4"/>
       <c r="D212" s="2" t="s">
         <v>443</v>
       </c>
@@ -17917,7 +17908,7 @@
       <c r="B213" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C213" s="5"/>
+      <c r="C213" s="4"/>
       <c r="D213" s="2" t="s">
         <v>445</v>
       </c>
@@ -17947,7 +17938,7 @@
       <c r="B214" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C214" s="5"/>
+      <c r="C214" s="4"/>
       <c r="D214" s="2" t="s">
         <v>447</v>
       </c>
@@ -17977,7 +17968,7 @@
       <c r="B215" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C215" s="5"/>
+      <c r="C215" s="4"/>
       <c r="D215" s="2" t="s">
         <v>449</v>
       </c>
@@ -18007,7 +17998,7 @@
       <c r="B216" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C216" s="5"/>
+      <c r="C216" s="4"/>
       <c r="D216" s="2" t="s">
         <v>451</v>
       </c>
@@ -18037,7 +18028,7 @@
       <c r="B217" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C217" s="5"/>
+      <c r="C217" s="4"/>
       <c r="D217" s="2" t="s">
         <v>453</v>
       </c>
@@ -18067,7 +18058,7 @@
       <c r="B218" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C218" s="5"/>
+      <c r="C218" s="4"/>
       <c r="D218" s="2" t="s">
         <v>455</v>
       </c>
@@ -18129,7 +18120,7 @@
       <c r="B220" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C220" s="5"/>
+      <c r="C220" s="4"/>
       <c r="D220" s="2" t="s">
         <v>459</v>
       </c>
@@ -18159,7 +18150,7 @@
       <c r="B221" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C221" s="5"/>
+      <c r="C221" s="4"/>
       <c r="D221" s="2" t="s">
         <v>461</v>
       </c>
@@ -18189,7 +18180,7 @@
       <c r="B222" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C222" s="5"/>
+      <c r="C222" s="4"/>
       <c r="D222" s="2" t="s">
         <v>463</v>
       </c>
@@ -18219,7 +18210,7 @@
       <c r="B223" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C223" s="5"/>
+      <c r="C223" s="4"/>
       <c r="D223" s="2" t="s">
         <v>465</v>
       </c>
@@ -18249,7 +18240,7 @@
       <c r="B224" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C224" s="5"/>
+      <c r="C224" s="4"/>
       <c r="D224" s="2" t="s">
         <v>467</v>
       </c>
@@ -18279,7 +18270,7 @@
       <c r="B225" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C225" s="5"/>
+      <c r="C225" s="4"/>
       <c r="D225" s="2" t="s">
         <v>469</v>
       </c>
@@ -18309,7 +18300,7 @@
       <c r="B226" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C226" s="5"/>
+      <c r="C226" s="4"/>
       <c r="D226" s="2" t="s">
         <v>471</v>
       </c>
@@ -18339,7 +18330,7 @@
       <c r="B227" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C227" s="5"/>
+      <c r="C227" s="4"/>
       <c r="D227" s="2" t="s">
         <v>473</v>
       </c>
@@ -18369,7 +18360,7 @@
       <c r="B228" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C228" s="5"/>
+      <c r="C228" s="4"/>
       <c r="D228" s="2" t="s">
         <v>475</v>
       </c>
@@ -18399,7 +18390,7 @@
       <c r="B229" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C229" s="5"/>
+      <c r="C229" s="4"/>
       <c r="D229" s="2" t="s">
         <v>477</v>
       </c>
@@ -18429,7 +18420,7 @@
       <c r="B230" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C230" s="5"/>
+      <c r="C230" s="4"/>
       <c r="D230" s="2" t="s">
         <v>479</v>
       </c>
@@ -18459,7 +18450,7 @@
       <c r="B231" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C231" s="5"/>
+      <c r="C231" s="4"/>
       <c r="D231" s="2" t="s">
         <v>481</v>
       </c>
@@ -18489,7 +18480,7 @@
       <c r="B232" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C232" s="5"/>
+      <c r="C232" s="4"/>
       <c r="D232" s="2" t="s">
         <v>483</v>
       </c>
@@ -18519,7 +18510,7 @@
       <c r="B233" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C233" s="5"/>
+      <c r="C233" s="4"/>
       <c r="D233" s="2" t="s">
         <v>486</v>
       </c>
@@ -18549,7 +18540,7 @@
       <c r="B234" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C234" s="5"/>
+      <c r="C234" s="4"/>
       <c r="D234" s="2" t="s">
         <v>488</v>
       </c>
@@ -18579,7 +18570,7 @@
       <c r="B235" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C235" s="5"/>
+      <c r="C235" s="4"/>
       <c r="D235" s="2" t="s">
         <v>490</v>
       </c>
@@ -18609,7 +18600,7 @@
       <c r="B236" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C236" s="5"/>
+      <c r="C236" s="4"/>
       <c r="D236" s="2" t="s">
         <v>492</v>
       </c>
@@ -18639,7 +18630,7 @@
       <c r="B237" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C237" s="5"/>
+      <c r="C237" s="4"/>
       <c r="D237" s="2" t="s">
         <v>494</v>
       </c>
@@ -18669,7 +18660,7 @@
       <c r="B238" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C238" s="5"/>
+      <c r="C238" s="4"/>
       <c r="D238" s="2" t="s">
         <v>496</v>
       </c>
@@ -18699,7 +18690,7 @@
       <c r="B239" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C239" s="5"/>
+      <c r="C239" s="4"/>
       <c r="D239" s="2" t="s">
         <v>498</v>
       </c>
@@ -18729,7 +18720,7 @@
       <c r="B240" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C240" s="5"/>
+      <c r="C240" s="4"/>
       <c r="D240" s="2" t="s">
         <v>501</v>
       </c>
@@ -18759,7 +18750,7 @@
       <c r="B241" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C241" s="5"/>
+      <c r="C241" s="4"/>
       <c r="D241" s="2" t="s">
         <v>502</v>
       </c>
@@ -18789,7 +18780,7 @@
       <c r="B242" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C242" s="5"/>
+      <c r="C242" s="4"/>
       <c r="D242" s="2" t="s">
         <v>503</v>
       </c>
@@ -18819,7 +18810,7 @@
       <c r="B243" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C243" s="5"/>
+      <c r="C243" s="4"/>
       <c r="D243" s="2" t="s">
         <v>505</v>
       </c>
@@ -18849,7 +18840,7 @@
       <c r="B244" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C244" s="5"/>
+      <c r="C244" s="4"/>
       <c r="D244" s="2" t="s">
         <v>507</v>
       </c>
@@ -18879,7 +18870,7 @@
       <c r="B245" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C245" s="5"/>
+      <c r="C245" s="4"/>
       <c r="D245" s="2" t="s">
         <v>508</v>
       </c>
@@ -18909,7 +18900,7 @@
       <c r="B246" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C246" s="5"/>
+      <c r="C246" s="4"/>
       <c r="D246" s="2" t="s">
         <v>510</v>
       </c>
@@ -18939,7 +18930,7 @@
       <c r="B247" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C247" s="5"/>
+      <c r="C247" s="4"/>
       <c r="D247" s="2" t="s">
         <v>512</v>
       </c>
@@ -18969,7 +18960,7 @@
       <c r="B248" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C248" s="5"/>
+      <c r="C248" s="4"/>
       <c r="D248" s="2" t="s">
         <v>514</v>
       </c>
@@ -18999,7 +18990,7 @@
       <c r="B249" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C249" s="5"/>
+      <c r="C249" s="4"/>
       <c r="D249" s="2" t="s">
         <v>516</v>
       </c>
@@ -19029,7 +19020,7 @@
       <c r="B250" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C250" s="5"/>
+      <c r="C250" s="4"/>
       <c r="D250" s="2" t="s">
         <v>518</v>
       </c>
@@ -19059,7 +19050,7 @@
       <c r="B251" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C251" s="5"/>
+      <c r="C251" s="4"/>
       <c r="D251" s="2" t="s">
         <v>520</v>
       </c>
@@ -19089,7 +19080,7 @@
       <c r="B252" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C252" s="5"/>
+      <c r="C252" s="4"/>
       <c r="D252" s="2" t="s">
         <v>522</v>
       </c>
@@ -19119,7 +19110,7 @@
       <c r="B253" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C253" s="5"/>
+      <c r="C253" s="4"/>
       <c r="D253" s="2" t="s">
         <v>524</v>
       </c>
@@ -19149,7 +19140,7 @@
       <c r="B254" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C254" s="5"/>
+      <c r="C254" s="4"/>
       <c r="D254" s="2" t="s">
         <v>526</v>
       </c>
@@ -19179,7 +19170,7 @@
       <c r="B255" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C255" s="5"/>
+      <c r="C255" s="4"/>
       <c r="D255" s="2" t="s">
         <v>528</v>
       </c>
@@ -19209,7 +19200,7 @@
       <c r="B256" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C256" s="5"/>
+      <c r="C256" s="4"/>
       <c r="D256" s="2" t="s">
         <v>530</v>
       </c>
@@ -19239,7 +19230,7 @@
       <c r="B257" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C257" s="5"/>
+      <c r="C257" s="4"/>
       <c r="D257" s="2" t="s">
         <v>532</v>
       </c>
@@ -19269,7 +19260,7 @@
       <c r="B258" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C258" s="5"/>
+      <c r="C258" s="4"/>
       <c r="D258" s="2" t="s">
         <v>534</v>
       </c>
@@ -19299,7 +19290,7 @@
       <c r="B259" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C259" s="5"/>
+      <c r="C259" s="4"/>
       <c r="D259" s="2" t="s">
         <v>536</v>
       </c>
@@ -19329,7 +19320,7 @@
       <c r="B260" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C260" s="5"/>
+      <c r="C260" s="4"/>
       <c r="D260" s="2" t="s">
         <v>538</v>
       </c>
@@ -19359,7 +19350,7 @@
       <c r="B261" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C261" s="5"/>
+      <c r="C261" s="4"/>
       <c r="D261" s="2" t="s">
         <v>540</v>
       </c>
@@ -19389,7 +19380,7 @@
       <c r="B262" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C262" s="5"/>
+      <c r="C262" s="4"/>
       <c r="D262" s="2" t="s">
         <v>542</v>
       </c>
@@ -19579,7 +19570,7 @@
       <c r="B268" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C268" s="5"/>
+      <c r="C268" s="4"/>
       <c r="D268" s="2" t="s">
         <v>555</v>
       </c>
@@ -19609,7 +19600,7 @@
       <c r="B269" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C269" s="5"/>
+      <c r="C269" s="4"/>
       <c r="D269" s="2" t="s">
         <v>557</v>
       </c>
@@ -19639,7 +19630,7 @@
       <c r="B270" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C270" s="5"/>
+      <c r="C270" s="4"/>
       <c r="D270" s="2" t="s">
         <v>559</v>
       </c>
@@ -19669,7 +19660,7 @@
       <c r="B271" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C271" s="5"/>
+      <c r="C271" s="4"/>
       <c r="D271" s="2" t="s">
         <v>561</v>
       </c>
@@ -19699,7 +19690,7 @@
       <c r="B272" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C272" s="5"/>
+      <c r="C272" s="4"/>
       <c r="D272" s="2" t="s">
         <v>563</v>
       </c>
@@ -19761,7 +19752,7 @@
       <c r="B274" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C274" s="5"/>
+      <c r="C274" s="4"/>
       <c r="D274" s="2" t="s">
         <v>567</v>
       </c>
@@ -19823,7 +19814,7 @@
       <c r="B276" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C276" s="5"/>
+      <c r="C276" s="4"/>
       <c r="D276" s="2" t="s">
         <v>571</v>
       </c>
@@ -19853,7 +19844,7 @@
       <c r="B277" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C277" s="5"/>
+      <c r="C277" s="4"/>
       <c r="D277" s="2" t="s">
         <v>574</v>
       </c>
@@ -19883,7 +19874,7 @@
       <c r="B278" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C278" s="5"/>
+      <c r="C278" s="4"/>
       <c r="D278" s="2" t="s">
         <v>576</v>
       </c>
@@ -19913,7 +19904,7 @@
       <c r="B279" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C279" s="5"/>
+      <c r="C279" s="4"/>
       <c r="D279" s="2" t="s">
         <v>578</v>
       </c>
@@ -19943,7 +19934,7 @@
       <c r="B280" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C280" s="5"/>
+      <c r="C280" s="4"/>
       <c r="D280" s="2" t="s">
         <v>580</v>
       </c>
@@ -19973,7 +19964,7 @@
       <c r="B281" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C281" s="4" t="s">
+      <c r="C281" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D281" s="2" t="s">
@@ -20005,7 +19996,7 @@
       <c r="B282" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C282" s="5"/>
+      <c r="C282" s="4"/>
       <c r="D282" s="2" t="s">
         <v>584</v>
       </c>
@@ -20675,7 +20666,7 @@
       <c r="B303" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C303" s="5"/>
+      <c r="C303" s="4"/>
       <c r="D303" s="2" t="s">
         <v>627</v>
       </c>
@@ -20993,7 +20984,7 @@
       <c r="B313" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C313" s="5"/>
+      <c r="C313" s="4"/>
       <c r="D313" s="2" t="s">
         <v>647</v>
       </c>
@@ -21599,7 +21590,7 @@
       <c r="B332" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C332" s="5"/>
+      <c r="C332" s="4"/>
       <c r="D332" s="2" t="s">
         <v>684</v>
       </c>
@@ -21629,7 +21620,7 @@
       <c r="B333" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C333" s="5"/>
+      <c r="C333" s="4"/>
       <c r="D333" s="2" t="s">
         <v>686</v>
       </c>
@@ -21659,7 +21650,7 @@
       <c r="B334" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C334" s="5"/>
+      <c r="C334" s="4"/>
       <c r="D334" s="2" t="s">
         <v>688</v>
       </c>
@@ -21689,7 +21680,7 @@
       <c r="B335" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C335" s="5"/>
+      <c r="C335" s="4"/>
       <c r="D335" s="2" t="s">
         <v>690</v>
       </c>
@@ -21719,7 +21710,7 @@
       <c r="B336" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C336" s="5"/>
+      <c r="C336" s="4"/>
       <c r="D336" s="2" t="s">
         <v>692</v>
       </c>
@@ -21749,7 +21740,7 @@
       <c r="B337" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C337" s="5"/>
+      <c r="C337" s="4"/>
       <c r="D337" s="2" t="s">
         <v>694</v>
       </c>
@@ -21875,7 +21866,7 @@
       <c r="B341" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C341" s="5"/>
+      <c r="C341" s="4"/>
       <c r="D341" s="2" t="s">
         <v>702</v>
       </c>
@@ -21905,7 +21896,7 @@
       <c r="B342" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C342" s="5"/>
+      <c r="C342" s="4"/>
       <c r="D342" s="2" t="s">
         <v>704</v>
       </c>
@@ -21935,7 +21926,7 @@
       <c r="B343" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C343" s="5"/>
+      <c r="C343" s="4"/>
       <c r="D343" s="2" t="s">
         <v>706</v>
       </c>
@@ -21965,7 +21956,7 @@
       <c r="B344" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C344" s="5"/>
+      <c r="C344" s="4"/>
       <c r="D344" s="2" t="s">
         <v>708</v>
       </c>
@@ -21995,7 +21986,7 @@
       <c r="B345" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C345" s="5"/>
+      <c r="C345" s="4"/>
       <c r="D345" s="2" t="s">
         <v>710</v>
       </c>
@@ -22025,7 +22016,7 @@
       <c r="B346" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C346" s="5"/>
+      <c r="C346" s="4"/>
       <c r="D346" s="2" t="s">
         <v>712</v>
       </c>
@@ -22055,7 +22046,7 @@
       <c r="B347" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C347" s="5"/>
+      <c r="C347" s="4"/>
       <c r="D347" s="2" t="s">
         <v>714</v>
       </c>
@@ -22085,7 +22076,7 @@
       <c r="B348" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C348" s="5"/>
+      <c r="C348" s="4"/>
       <c r="D348" s="2" t="s">
         <v>716</v>
       </c>
@@ -22115,7 +22106,7 @@
       <c r="B349" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C349" s="5"/>
+      <c r="C349" s="4"/>
       <c r="D349" s="2" t="s">
         <v>718</v>
       </c>
@@ -22145,7 +22136,7 @@
       <c r="B350" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C350" s="5"/>
+      <c r="C350" s="4"/>
       <c r="D350" s="2" t="s">
         <v>719</v>
       </c>
@@ -22175,7 +22166,7 @@
       <c r="B351" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C351" s="5"/>
+      <c r="C351" s="4"/>
       <c r="D351" s="2" t="s">
         <v>721</v>
       </c>
@@ -22205,7 +22196,7 @@
       <c r="B352" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C352" s="5"/>
+      <c r="C352" s="4"/>
       <c r="D352" s="2" t="s">
         <v>723</v>
       </c>
@@ -22235,7 +22226,7 @@
       <c r="B353" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C353" s="5"/>
+      <c r="C353" s="4"/>
       <c r="D353" s="2" t="s">
         <v>725</v>
       </c>
@@ -22265,7 +22256,7 @@
       <c r="B354" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C354" s="5"/>
+      <c r="C354" s="4"/>
       <c r="D354" s="2" t="s">
         <v>727</v>
       </c>
@@ -22295,7 +22286,7 @@
       <c r="B355" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C355" s="5"/>
+      <c r="C355" s="4"/>
       <c r="D355" s="2" t="s">
         <v>729</v>
       </c>
@@ -22325,7 +22316,7 @@
       <c r="B356" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C356" s="5"/>
+      <c r="C356" s="4"/>
       <c r="D356" s="2" t="s">
         <v>731</v>
       </c>
@@ -22355,7 +22346,7 @@
       <c r="B357" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C357" s="5"/>
+      <c r="C357" s="4"/>
       <c r="D357" s="2" t="s">
         <v>733</v>
       </c>
@@ -22385,7 +22376,7 @@
       <c r="B358" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C358" s="5"/>
+      <c r="C358" s="4"/>
       <c r="D358" s="2" t="s">
         <v>735</v>
       </c>
@@ -22415,7 +22406,7 @@
       <c r="B359" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C359" s="5"/>
+      <c r="C359" s="4"/>
       <c r="D359" s="2" t="s">
         <v>737</v>
       </c>
@@ -22765,7 +22756,7 @@
       <c r="B370" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C370" s="5"/>
+      <c r="C370" s="4"/>
       <c r="D370" s="2" t="s">
         <v>758</v>
       </c>
@@ -22795,7 +22786,7 @@
       <c r="B371" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C371" s="5"/>
+      <c r="C371" s="4"/>
       <c r="D371" s="2" t="s">
         <v>760</v>
       </c>
@@ -22825,7 +22816,7 @@
       <c r="B372" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C372" s="5"/>
+      <c r="C372" s="4"/>
       <c r="D372" s="2" t="s">
         <v>762</v>
       </c>
@@ -22887,7 +22878,7 @@
       <c r="B374" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C374" s="5"/>
+      <c r="C374" s="4"/>
       <c r="D374" s="2" t="s">
         <v>766</v>
       </c>
@@ -23013,7 +23004,7 @@
       <c r="B378" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C378" s="5"/>
+      <c r="C378" s="4"/>
       <c r="D378" s="2" t="s">
         <v>774</v>
       </c>
@@ -23075,7 +23066,7 @@
       <c r="B380" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C380" s="5"/>
+      <c r="C380" s="4"/>
       <c r="D380" s="2" t="s">
         <v>778</v>
       </c>
@@ -23137,7 +23128,7 @@
       <c r="B382" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C382" s="5"/>
+      <c r="C382" s="4"/>
       <c r="D382" s="2" t="s">
         <v>782</v>
       </c>
@@ -23167,7 +23158,7 @@
       <c r="B383" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C383" s="5"/>
+      <c r="C383" s="4"/>
       <c r="D383" s="2" t="s">
         <v>784</v>
       </c>
@@ -23197,7 +23188,7 @@
       <c r="B384" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C384" s="5"/>
+      <c r="C384" s="4"/>
       <c r="D384" s="2" t="s">
         <v>786</v>
       </c>
@@ -23227,7 +23218,7 @@
       <c r="B385" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C385" s="5"/>
+      <c r="C385" s="4"/>
       <c r="D385" s="2" t="s">
         <v>788</v>
       </c>
@@ -23257,7 +23248,7 @@
       <c r="B386" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C386" s="5"/>
+      <c r="C386" s="4"/>
       <c r="D386" s="2" t="s">
         <v>790</v>
       </c>
@@ -23287,7 +23278,7 @@
       <c r="B387" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C387" s="5"/>
+      <c r="C387" s="4"/>
       <c r="D387" s="2" t="s">
         <v>792</v>
       </c>
@@ -23317,7 +23308,7 @@
       <c r="B388" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C388" s="5"/>
+      <c r="C388" s="4"/>
       <c r="D388" s="2" t="s">
         <v>794</v>
       </c>
@@ -23347,7 +23338,7 @@
       <c r="B389" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C389" s="5"/>
+      <c r="C389" s="4"/>
       <c r="D389" s="2" t="s">
         <v>795</v>
       </c>
@@ -23377,7 +23368,7 @@
       <c r="B390" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C390" s="5"/>
+      <c r="C390" s="4"/>
       <c r="D390" s="2" t="s">
         <v>796</v>
       </c>
@@ -23407,7 +23398,7 @@
       <c r="B391" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C391" s="5"/>
+      <c r="C391" s="4"/>
       <c r="D391" s="2" t="s">
         <v>797</v>
       </c>
@@ -23437,7 +23428,7 @@
       <c r="B392" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C392" s="5"/>
+      <c r="C392" s="4"/>
       <c r="D392" s="2" t="s">
         <v>799</v>
       </c>
@@ -23627,7 +23618,7 @@
       <c r="B398" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C398" s="5"/>
+      <c r="C398" s="4"/>
       <c r="D398" s="2" t="s">
         <v>811</v>
       </c>
@@ -23657,7 +23648,7 @@
       <c r="B399" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C399" s="5"/>
+      <c r="C399" s="4"/>
       <c r="D399" s="2" t="s">
         <v>814</v>
       </c>
@@ -23687,7 +23678,7 @@
       <c r="B400" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C400" s="5"/>
+      <c r="C400" s="4"/>
       <c r="D400" s="2" t="s">
         <v>816</v>
       </c>
@@ -23717,7 +23708,7 @@
       <c r="B401" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C401" s="5"/>
+      <c r="C401" s="4"/>
       <c r="D401" s="2" t="s">
         <v>817</v>
       </c>
@@ -23747,7 +23738,7 @@
       <c r="B402" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C402" s="5"/>
+      <c r="C402" s="4"/>
       <c r="D402" s="2" t="s">
         <v>819</v>
       </c>
@@ -23809,7 +23800,7 @@
       <c r="B404" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C404" s="5"/>
+      <c r="C404" s="4"/>
       <c r="D404" s="2" t="s">
         <v>823</v>
       </c>
@@ -23839,7 +23830,7 @@
       <c r="B405" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C405" s="5"/>
+      <c r="C405" s="4"/>
       <c r="D405" s="2" t="s">
         <v>825</v>
       </c>
@@ -23869,7 +23860,7 @@
       <c r="B406" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C406" s="5"/>
+      <c r="C406" s="4"/>
       <c r="D406" s="2" t="s">
         <v>827</v>
       </c>
@@ -23899,7 +23890,7 @@
       <c r="B407" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C407" s="5"/>
+      <c r="C407" s="4"/>
       <c r="D407" s="2" t="s">
         <v>829</v>
       </c>
@@ -23929,7 +23920,7 @@
       <c r="B408" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C408" s="5"/>
+      <c r="C408" s="4"/>
       <c r="D408" s="2" t="s">
         <v>831</v>
       </c>
@@ -23991,7 +23982,7 @@
       <c r="B410" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C410" s="5"/>
+      <c r="C410" s="4"/>
       <c r="D410" s="2" t="s">
         <v>836</v>
       </c>
@@ -24309,7 +24300,7 @@
       <c r="B420" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C420" s="5"/>
+      <c r="C420" s="4"/>
       <c r="D420" s="2" t="s">
         <v>856</v>
       </c>
@@ -25203,7 +25194,7 @@
       <c r="B448" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C448" s="5"/>
+      <c r="C448" s="4"/>
       <c r="D448" s="2" t="s">
         <v>912</v>
       </c>
@@ -25649,7 +25640,7 @@
       <c r="B462" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C462" s="5"/>
+      <c r="C462" s="4"/>
       <c r="D462" s="2" t="s">
         <v>940</v>
       </c>
@@ -25679,7 +25670,7 @@
       <c r="B463" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C463" s="5"/>
+      <c r="C463" s="4"/>
       <c r="D463" s="2" t="s">
         <v>942</v>
       </c>
@@ -25709,7 +25700,7 @@
       <c r="B464" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C464" s="5"/>
+      <c r="C464" s="4"/>
       <c r="D464" s="2" t="s">
         <v>944</v>
       </c>
@@ -26187,7 +26178,7 @@
       <c r="B479" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C479" s="4" t="s">
+      <c r="C479" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D479" s="2" t="s">
@@ -26443,7 +26434,7 @@
       <c r="B487" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C487" s="5"/>
+      <c r="C487" s="4"/>
       <c r="D487" s="2" t="s">
         <v>990</v>
       </c>
@@ -26569,7 +26560,7 @@
       <c r="B491" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C491" s="5"/>
+      <c r="C491" s="4"/>
       <c r="D491" s="2" t="s">
         <v>997</v>
       </c>
@@ -26599,7 +26590,7 @@
       <c r="B492" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C492" s="5"/>
+      <c r="C492" s="4"/>
       <c r="D492" s="2" t="s">
         <v>999</v>
       </c>
@@ -27077,7 +27068,7 @@
       <c r="B507" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C507" s="5"/>
+      <c r="C507" s="4"/>
       <c r="D507" s="2" t="s">
         <v>1029</v>
       </c>
@@ -27139,7 +27130,7 @@
       <c r="B509" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C509" s="4" t="s">
+      <c r="C509" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D509" s="2" t="s">
@@ -27523,7 +27514,7 @@
       <c r="B521" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C521" s="5"/>
+      <c r="C521" s="4"/>
       <c r="D521" s="2" t="s">
         <v>1056</v>
       </c>
@@ -27553,7 +27544,7 @@
       <c r="B522" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C522" s="5"/>
+      <c r="C522" s="4"/>
       <c r="D522" s="2" t="s">
         <v>1058</v>
       </c>
@@ -27583,7 +27574,7 @@
       <c r="B523" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C523" s="5"/>
+      <c r="C523" s="4"/>
       <c r="D523" s="2" t="s">
         <v>1060</v>
       </c>
@@ -27645,7 +27636,7 @@
       <c r="B525" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C525" s="5"/>
+      <c r="C525" s="4"/>
       <c r="D525" s="2" t="s">
         <v>1064</v>
       </c>
@@ -27707,7 +27698,7 @@
       <c r="B527" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C527" s="5"/>
+      <c r="C527" s="4"/>
       <c r="D527" s="2" t="s">
         <v>1068</v>
       </c>
@@ -27769,7 +27760,7 @@
       <c r="B529" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C529" s="5"/>
+      <c r="C529" s="4"/>
       <c r="D529" s="2" t="s">
         <v>1072</v>
       </c>
@@ -27799,7 +27790,7 @@
       <c r="B530" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C530" s="5"/>
+      <c r="C530" s="4"/>
       <c r="D530" s="2" t="s">
         <v>1074</v>
       </c>
@@ -27829,7 +27820,7 @@
       <c r="B531" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C531" s="5"/>
+      <c r="C531" s="4"/>
       <c r="D531" s="2" t="s">
         <v>1076</v>
       </c>
@@ -27859,7 +27850,7 @@
       <c r="B532" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C532" s="5"/>
+      <c r="C532" s="4"/>
       <c r="D532" s="2" t="s">
         <v>1078</v>
       </c>
@@ -27889,7 +27880,7 @@
       <c r="B533" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C533" s="5"/>
+      <c r="C533" s="4"/>
       <c r="D533" s="2" t="s">
         <v>1080</v>
       </c>
@@ -27983,7 +27974,7 @@
       <c r="B536" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C536" s="5"/>
+      <c r="C536" s="4"/>
       <c r="D536" s="2" t="s">
         <v>1086</v>
       </c>
@@ -28045,7 +28036,7 @@
       <c r="B538" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C538" s="5"/>
+      <c r="C538" s="4"/>
       <c r="D538" s="2" t="s">
         <v>1090</v>
       </c>
@@ -28075,7 +28066,7 @@
       <c r="B539" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C539" s="5"/>
+      <c r="C539" s="4"/>
       <c r="D539" s="2" t="s">
         <v>1092</v>
       </c>
@@ -28105,7 +28096,7 @@
       <c r="B540" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C540" s="5"/>
+      <c r="C540" s="4"/>
       <c r="D540" s="2" t="s">
         <v>1094</v>
       </c>
@@ -28295,7 +28286,7 @@
       <c r="B546" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C546" s="5"/>
+      <c r="C546" s="4"/>
       <c r="D546" s="2" t="s">
         <v>1105</v>
       </c>
@@ -28325,7 +28316,7 @@
       <c r="B547" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C547" s="5"/>
+      <c r="C547" s="4"/>
       <c r="D547" s="2" t="s">
         <v>1107</v>
       </c>
@@ -28355,7 +28346,7 @@
       <c r="B548" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C548" s="5"/>
+      <c r="C548" s="4"/>
       <c r="D548" s="2" t="s">
         <v>1109</v>
       </c>
@@ -28417,7 +28408,7 @@
       <c r="B550" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C550" s="5"/>
+      <c r="C550" s="4"/>
       <c r="D550" s="2" t="s">
         <v>1113</v>
       </c>
@@ -28447,7 +28438,7 @@
       <c r="B551" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C551" s="5"/>
+      <c r="C551" s="4"/>
       <c r="D551" s="2" t="s">
         <v>1115</v>
       </c>
@@ -28477,7 +28468,7 @@
       <c r="B552" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C552" s="5"/>
+      <c r="C552" s="4"/>
       <c r="D552" s="2" t="s">
         <v>1117</v>
       </c>
@@ -28507,7 +28498,7 @@
       <c r="B553" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C553" s="5"/>
+      <c r="C553" s="4"/>
       <c r="D553" s="2" t="s">
         <v>1119</v>
       </c>
@@ -28537,7 +28528,7 @@
       <c r="B554" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C554" s="5"/>
+      <c r="C554" s="4"/>
       <c r="D554" s="2" t="s">
         <v>1121</v>
       </c>
@@ -28567,7 +28558,7 @@
       <c r="B555" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C555" s="5"/>
+      <c r="C555" s="4"/>
       <c r="D555" s="2" t="s">
         <v>1123</v>
       </c>
@@ -28597,7 +28588,7 @@
       <c r="B556" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C556" s="5"/>
+      <c r="C556" s="4"/>
       <c r="D556" s="2" t="s">
         <v>1125</v>
       </c>
@@ -28627,7 +28618,7 @@
       <c r="B557" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C557" s="5"/>
+      <c r="C557" s="4"/>
       <c r="D557" s="2" t="s">
         <v>1127</v>
       </c>
@@ -28657,7 +28648,7 @@
       <c r="B558" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C558" s="5"/>
+      <c r="C558" s="4"/>
       <c r="D558" s="2" t="s">
         <v>1129</v>
       </c>
@@ -28687,7 +28678,7 @@
       <c r="B559" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C559" s="5"/>
+      <c r="C559" s="4"/>
       <c r="D559" s="2" t="s">
         <v>1131</v>
       </c>
@@ -29325,7 +29316,7 @@
       <c r="B579" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C579" s="5"/>
+      <c r="C579" s="4"/>
       <c r="D579" s="2" t="s">
         <v>1171</v>
       </c>
@@ -29355,7 +29346,7 @@
       <c r="B580" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C580" s="5"/>
+      <c r="C580" s="4"/>
       <c r="D580" s="2" t="s">
         <v>1173</v>
       </c>
@@ -29385,7 +29376,7 @@
       <c r="B581" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C581" s="5"/>
+      <c r="C581" s="4"/>
       <c r="D581" s="2" t="s">
         <v>1175</v>
       </c>
@@ -29415,7 +29406,7 @@
       <c r="B582" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C582" s="5"/>
+      <c r="C582" s="4"/>
       <c r="D582" s="2" t="s">
         <v>1177</v>
       </c>
@@ -29445,7 +29436,7 @@
       <c r="B583" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C583" s="5"/>
+      <c r="C583" s="4"/>
       <c r="D583" s="2" t="s">
         <v>1179</v>
       </c>
@@ -29475,7 +29466,7 @@
       <c r="B584" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C584" s="5"/>
+      <c r="C584" s="4"/>
       <c r="D584" s="2" t="s">
         <v>1181</v>
       </c>
@@ -29505,7 +29496,7 @@
       <c r="B585" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C585" s="5"/>
+      <c r="C585" s="4"/>
       <c r="D585" s="2" t="s">
         <v>1183</v>
       </c>
@@ -29535,7 +29526,7 @@
       <c r="B586" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C586" s="5"/>
+      <c r="C586" s="4"/>
       <c r="D586" s="2" t="s">
         <v>1185</v>
       </c>
@@ -29565,7 +29556,7 @@
       <c r="B587" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C587" s="5"/>
+      <c r="C587" s="4"/>
       <c r="D587" s="2" t="s">
         <v>1187</v>
       </c>
@@ -29595,7 +29586,7 @@
       <c r="B588" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C588" s="5"/>
+      <c r="C588" s="4"/>
       <c r="D588" s="2" t="s">
         <v>1189</v>
       </c>
@@ -29625,7 +29616,7 @@
       <c r="B589" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C589" s="5"/>
+      <c r="C589" s="4"/>
       <c r="D589" s="2" t="s">
         <v>1191</v>
       </c>
@@ -29655,7 +29646,7 @@
       <c r="B590" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C590" s="5"/>
+      <c r="C590" s="4"/>
       <c r="D590" s="2" t="s">
         <v>1193</v>
       </c>
@@ -29685,7 +29676,7 @@
       <c r="B591" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C591" s="5"/>
+      <c r="C591" s="4"/>
       <c r="D591" s="2" t="s">
         <v>1195</v>
       </c>
@@ -29715,7 +29706,7 @@
       <c r="B592" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C592" s="5"/>
+      <c r="C592" s="4"/>
       <c r="D592" s="2" t="s">
         <v>1197</v>
       </c>
@@ -29745,7 +29736,7 @@
       <c r="B593" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C593" s="5"/>
+      <c r="C593" s="4"/>
       <c r="D593" s="2" t="s">
         <v>1199</v>
       </c>
@@ -29775,7 +29766,7 @@
       <c r="B594" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C594" s="5"/>
+      <c r="C594" s="4"/>
       <c r="D594" s="2" t="s">
         <v>1201</v>
       </c>
@@ -29837,7 +29828,7 @@
       <c r="B596" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C596" s="5"/>
+      <c r="C596" s="4"/>
       <c r="D596" s="2" t="s">
         <v>1205</v>
       </c>
@@ -29995,7 +29986,7 @@
       <c r="B601" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C601" s="5"/>
+      <c r="C601" s="4"/>
       <c r="D601" s="2" t="s">
         <v>1216</v>
       </c>
@@ -30057,7 +30048,7 @@
       <c r="B603" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C603" s="5"/>
+      <c r="C603" s="4"/>
       <c r="D603" s="2" t="s">
         <v>1221</v>
       </c>
@@ -30087,7 +30078,7 @@
       <c r="B604" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C604" s="5"/>
+      <c r="C604" s="4"/>
       <c r="D604" s="2" t="s">
         <v>1223</v>
       </c>
@@ -30117,7 +30108,7 @@
       <c r="B605" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C605" s="5"/>
+      <c r="C605" s="4"/>
       <c r="D605" s="2" t="s">
         <v>1225</v>
       </c>
@@ -30179,7 +30170,7 @@
       <c r="B607" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C607" s="5"/>
+      <c r="C607" s="4"/>
       <c r="D607" s="2" t="s">
         <v>1229</v>
       </c>
@@ -30241,7 +30232,7 @@
       <c r="B609" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C609" s="5"/>
+      <c r="C609" s="4"/>
       <c r="D609" s="2" t="s">
         <v>1233</v>
       </c>
@@ -30271,7 +30262,7 @@
       <c r="B610" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C610" s="5"/>
+      <c r="C610" s="4"/>
       <c r="D610" s="2" t="s">
         <v>1235</v>
       </c>
@@ -31517,7 +31508,7 @@
       <c r="B649" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C649" s="5"/>
+      <c r="C649" s="4"/>
       <c r="D649" s="2" t="s">
         <v>1313</v>
       </c>
@@ -31547,7 +31538,7 @@
       <c r="B650" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C650" s="5"/>
+      <c r="C650" s="4"/>
       <c r="D650" s="2" t="s">
         <v>1315</v>
       </c>
@@ -31737,7 +31728,7 @@
       <c r="B656" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C656" s="5"/>
+      <c r="C656" s="4"/>
       <c r="D656" s="2" t="s">
         <v>1328</v>
       </c>
@@ -31767,7 +31758,7 @@
       <c r="B657" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C657" s="5"/>
+      <c r="C657" s="4"/>
       <c r="D657" s="2" t="s">
         <v>1330</v>
       </c>
@@ -31797,7 +31788,7 @@
       <c r="B658" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C658" s="5"/>
+      <c r="C658" s="4"/>
       <c r="D658" s="2" t="s">
         <v>1332</v>
       </c>
@@ -31827,7 +31818,7 @@
       <c r="B659" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C659" s="5"/>
+      <c r="C659" s="4"/>
       <c r="D659" s="2" t="s">
         <v>1334</v>
       </c>
@@ -31857,7 +31848,7 @@
       <c r="B660" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C660" s="5"/>
+      <c r="C660" s="4"/>
       <c r="D660" s="2" t="s">
         <v>1336</v>
       </c>
@@ -31887,7 +31878,7 @@
       <c r="B661" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C661" s="5"/>
+      <c r="C661" s="4"/>
       <c r="D661" s="2" t="s">
         <v>1338</v>
       </c>
@@ -31917,7 +31908,7 @@
       <c r="B662" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C662" s="5"/>
+      <c r="C662" s="4"/>
       <c r="D662" s="2" t="s">
         <v>1340</v>
       </c>
@@ -31947,7 +31938,7 @@
       <c r="B663" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C663" s="5"/>
+      <c r="C663" s="4"/>
       <c r="D663" s="2" t="s">
         <v>1342</v>
       </c>
@@ -31977,7 +31968,7 @@
       <c r="B664" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C664" s="5"/>
+      <c r="C664" s="4"/>
       <c r="D664" s="2" t="s">
         <v>1344</v>
       </c>
@@ -32007,7 +31998,7 @@
       <c r="B665" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C665" s="5"/>
+      <c r="C665" s="4"/>
       <c r="D665" s="2" t="s">
         <v>1346</v>
       </c>
@@ -32037,7 +32028,7 @@
       <c r="B666" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C666" s="5"/>
+      <c r="C666" s="4"/>
       <c r="D666" s="2" t="s">
         <v>1348</v>
       </c>
@@ -32067,7 +32058,7 @@
       <c r="B667" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C667" s="5"/>
+      <c r="C667" s="4"/>
       <c r="D667" s="2" t="s">
         <v>1350</v>
       </c>
@@ -32097,7 +32088,7 @@
       <c r="B668" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C668" s="5"/>
+      <c r="C668" s="4"/>
       <c r="D668" s="2" t="s">
         <v>1352</v>
       </c>
@@ -32127,7 +32118,7 @@
       <c r="B669" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C669" s="5"/>
+      <c r="C669" s="4"/>
       <c r="D669" s="2" t="s">
         <v>1354</v>
       </c>
@@ -32157,7 +32148,7 @@
       <c r="B670" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C670" s="5"/>
+      <c r="C670" s="4"/>
       <c r="D670" s="2" t="s">
         <v>1356</v>
       </c>
@@ -32187,7 +32178,7 @@
       <c r="B671" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C671" s="5"/>
+      <c r="C671" s="4"/>
       <c r="D671" s="2" t="s">
         <v>1358</v>
       </c>
@@ -33433,7 +33424,7 @@
       <c r="B710" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C710" s="4" t="s">
+      <c r="C710" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D710" s="2" t="s">
@@ -34425,7 +34416,7 @@
       <c r="B741" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C741" s="5"/>
+      <c r="C741" s="4"/>
       <c r="D741" s="2" t="s">
         <v>1499</v>
       </c>
@@ -34807,7 +34798,7 @@
       <c r="B753" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C753" s="5"/>
+      <c r="C753" s="4"/>
       <c r="D753" s="2" t="s">
         <v>1524</v>
       </c>
@@ -34837,7 +34828,7 @@
       <c r="B754" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C754" s="5"/>
+      <c r="C754" s="4"/>
       <c r="D754" s="2" t="s">
         <v>1527</v>
       </c>
@@ -36019,7 +36010,7 @@
       <c r="B791" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C791" s="4" t="s">
+      <c r="C791" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D791" s="2" t="s">
@@ -36371,7 +36362,7 @@
       <c r="B802" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C802" s="5"/>
+      <c r="C802" s="4"/>
       <c r="D802" s="2" t="s">
         <v>1624</v>
       </c>
@@ -37521,7 +37512,7 @@
       <c r="B838" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C838" s="5"/>
+      <c r="C838" s="4"/>
       <c r="D838" s="2" t="s">
         <v>1696</v>
       </c>
@@ -37551,7 +37542,7 @@
       <c r="B839" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C839" s="5"/>
+      <c r="C839" s="4"/>
       <c r="D839" s="2" t="s">
         <v>1698</v>
       </c>
@@ -37581,7 +37572,7 @@
       <c r="B840" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C840" s="5"/>
+      <c r="C840" s="4"/>
       <c r="D840" s="2" t="s">
         <v>1700</v>
       </c>
@@ -37611,7 +37602,7 @@
       <c r="B841" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C841" s="5"/>
+      <c r="C841" s="4"/>
       <c r="D841" s="2" t="s">
         <v>1702</v>
       </c>
@@ -37641,7 +37632,7 @@
       <c r="B842" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C842" s="5"/>
+      <c r="C842" s="4"/>
       <c r="D842" s="2" t="s">
         <v>1704</v>
       </c>
@@ -37671,7 +37662,7 @@
       <c r="B843" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C843" s="5"/>
+      <c r="C843" s="4"/>
       <c r="D843" s="2" t="s">
         <v>1706</v>
       </c>
@@ -37701,7 +37692,7 @@
       <c r="B844" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C844" s="5"/>
+      <c r="C844" s="4"/>
       <c r="D844" s="2" t="s">
         <v>1708</v>
       </c>
@@ -37731,7 +37722,7 @@
       <c r="B845" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C845" s="5"/>
+      <c r="C845" s="4"/>
       <c r="D845" s="2" t="s">
         <v>1710</v>
       </c>
@@ -37761,7 +37752,7 @@
       <c r="B846" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C846" s="5"/>
+      <c r="C846" s="4"/>
       <c r="D846" s="2" t="s">
         <v>1712</v>
       </c>
@@ -37791,7 +37782,7 @@
       <c r="B847" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C847" s="5"/>
+      <c r="C847" s="4"/>
       <c r="D847" s="2" t="s">
         <v>1714</v>
       </c>
@@ -37821,7 +37812,7 @@
       <c r="B848" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C848" s="5"/>
+      <c r="C848" s="4"/>
       <c r="D848" s="2" t="s">
         <v>1716</v>
       </c>
@@ -37851,7 +37842,7 @@
       <c r="B849" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C849" s="5"/>
+      <c r="C849" s="4"/>
       <c r="D849" s="2" t="s">
         <v>1718</v>
       </c>
@@ -37881,7 +37872,7 @@
       <c r="B850" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C850" s="5"/>
+      <c r="C850" s="4"/>
       <c r="D850" s="2" t="s">
         <v>1720</v>
       </c>
@@ -37911,7 +37902,7 @@
       <c r="B851" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C851" s="5"/>
+      <c r="C851" s="4"/>
       <c r="D851" s="2" t="s">
         <v>1722</v>
       </c>
@@ -37941,7 +37932,7 @@
       <c r="B852" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C852" s="5"/>
+      <c r="C852" s="4"/>
       <c r="D852" s="2" t="s">
         <v>1724</v>
       </c>
@@ -38003,7 +37994,7 @@
       <c r="B854" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C854" s="5"/>
+      <c r="C854" s="4"/>
       <c r="D854" s="2" t="s">
         <v>1728</v>
       </c>
@@ -38065,7 +38056,7 @@
       <c r="B856" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C856" s="5"/>
+      <c r="C856" s="4"/>
       <c r="D856" s="2" t="s">
         <v>1732</v>
       </c>
@@ -38127,7 +38118,7 @@
       <c r="B858" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C858" s="5"/>
+      <c r="C858" s="4"/>
       <c r="D858" s="2" t="s">
         <v>1736</v>
       </c>
@@ -38189,7 +38180,7 @@
       <c r="B860" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C860" s="5"/>
+      <c r="C860" s="4"/>
       <c r="D860" s="2" t="s">
         <v>1740</v>
       </c>
@@ -39723,7 +39714,7 @@
       <c r="B908" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C908" s="5"/>
+      <c r="C908" s="4"/>
       <c r="D908" s="2" t="s">
         <v>1836</v>
       </c>
@@ -43561,7 +43552,7 @@
       <c r="B1028" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1028" s="4" t="s">
+      <c r="C1028" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1028" s="2" t="s">
@@ -47241,7 +47232,7 @@
       <c r="B1143" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1143" s="4" t="s">
+      <c r="C1143" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1143" s="2" t="s">
@@ -47849,7 +47840,7 @@
       <c r="B1162" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1162" s="4" t="s">
+      <c r="C1162" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1162" s="2" t="s">
@@ -49929,7 +49920,7 @@
       <c r="B1227" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C1227" s="5"/>
+      <c r="C1227" s="4"/>
       <c r="D1227" s="2" t="s">
         <v>2472</v>
       </c>
@@ -49959,7 +49950,7 @@
       <c r="B1228" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C1228" s="5"/>
+      <c r="C1228" s="4"/>
       <c r="D1228" s="2" t="s">
         <v>2474</v>
       </c>
@@ -49989,7 +49980,7 @@
       <c r="B1229" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C1229" s="5"/>
+      <c r="C1229" s="4"/>
       <c r="D1229" s="2" t="s">
         <v>2476</v>
       </c>
@@ -50051,7 +50042,7 @@
       <c r="B1231" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="C1231" s="5"/>
+      <c r="C1231" s="4"/>
       <c r="D1231" s="2" t="s">
         <v>2480</v>
       </c>
@@ -50081,7 +50072,7 @@
       <c r="B1232" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C1232" s="5"/>
+      <c r="C1232" s="4"/>
       <c r="D1232" s="2" t="s">
         <v>2482</v>
       </c>
@@ -50111,7 +50102,7 @@
       <c r="B1233" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C1233" s="5"/>
+      <c r="C1233" s="4"/>
       <c r="D1233" s="2" t="s">
         <v>2484</v>
       </c>
@@ -50781,7 +50772,7 @@
       <c r="B1254" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1254" s="4" t="s">
+      <c r="C1254" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1254" s="2" t="s">
@@ -52509,7 +52500,7 @@
       <c r="B1308" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1308" s="4" t="s">
+      <c r="C1308" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1308" s="2" t="s">
@@ -53405,7 +53396,7 @@
       <c r="B1336" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1336" s="4" t="s">
+      <c r="C1336" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1336" s="2" t="s">
@@ -53885,7 +53876,7 @@
       <c r="B1351" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1351" s="4" t="s">
+      <c r="C1351" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1351" s="2" t="s">
@@ -54781,7 +54772,7 @@
       <c r="B1379" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1379" s="4" t="s">
+      <c r="C1379" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1379" s="2" t="s">
@@ -55453,7 +55444,7 @@
       <c r="B1400" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1400" s="4" t="s">
+      <c r="C1400" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1400" s="2" t="s">
@@ -56125,7 +56116,7 @@
       <c r="B1421" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1421" s="4" t="s">
+      <c r="C1421" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1421" s="2" t="s">
@@ -56797,7 +56788,7 @@
       <c r="B1442" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1442" s="4" t="s">
+      <c r="C1442" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1442" s="2" t="s">
@@ -57469,7 +57460,7 @@
       <c r="B1463" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1463" s="4" t="s">
+      <c r="C1463" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1463" s="2" t="s">
@@ -58397,7 +58388,7 @@
       <c r="B1492" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1492" s="4" t="s">
+      <c r="C1492" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1492" s="2" t="s">
@@ -59357,7 +59348,7 @@
       <c r="B1522" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1522" s="4" t="s">
+      <c r="C1522" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1522" s="2" t="s">
@@ -60317,7 +60308,7 @@
       <c r="B1552" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1552" s="4" t="s">
+      <c r="C1552" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1552" s="2" t="s">
@@ -61277,7 +61268,7 @@
       <c r="B1582" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1582" s="4" t="s">
+      <c r="C1582" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1582" s="2" t="s">
@@ -62973,7 +62964,7 @@
       <c r="B1635" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1635" s="4" t="s">
+      <c r="C1635" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1635" s="2" t="s">
@@ -65181,7 +65172,7 @@
       <c r="B1704" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1704" s="5"/>
+      <c r="C1704" s="4"/>
       <c r="D1704" s="2" t="s">
         <v>3428</v>
       </c>
@@ -65211,7 +65202,7 @@
       <c r="B1705" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1705" s="5"/>
+      <c r="C1705" s="4"/>
       <c r="D1705" s="2" t="s">
         <v>3430</v>
       </c>
@@ -65241,7 +65232,7 @@
       <c r="B1706" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1706" s="5"/>
+      <c r="C1706" s="4"/>
       <c r="D1706" s="2" t="s">
         <v>3432</v>
       </c>
@@ -65271,7 +65262,7 @@
       <c r="B1707" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1707" s="5"/>
+      <c r="C1707" s="4"/>
       <c r="D1707" s="2" t="s">
         <v>3435</v>
       </c>
@@ -65301,7 +65292,7 @@
       <c r="B1708" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1708" s="5"/>
+      <c r="C1708" s="4"/>
       <c r="D1708" s="2" t="s">
         <v>3437</v>
       </c>
@@ -65331,7 +65322,7 @@
       <c r="B1709" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1709" s="5"/>
+      <c r="C1709" s="4"/>
       <c r="D1709" s="2" t="s">
         <v>3439</v>
       </c>
@@ -65361,7 +65352,7 @@
       <c r="B1710" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1710" s="5"/>
+      <c r="C1710" s="4"/>
       <c r="D1710" s="2" t="s">
         <v>3441</v>
       </c>
@@ -65391,7 +65382,7 @@
       <c r="B1711" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1711" s="5"/>
+      <c r="C1711" s="4"/>
       <c r="D1711" s="2" t="s">
         <v>3443</v>
       </c>
@@ -65421,7 +65412,7 @@
       <c r="B1712" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1712" s="5"/>
+      <c r="C1712" s="4"/>
       <c r="D1712" s="2" t="s">
         <v>3445</v>
       </c>
@@ -65451,7 +65442,7 @@
       <c r="B1713" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1713" s="5"/>
+      <c r="C1713" s="4"/>
       <c r="D1713" s="2" t="s">
         <v>3447</v>
       </c>
@@ -65481,7 +65472,7 @@
       <c r="B1714" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1714" s="5"/>
+      <c r="C1714" s="4"/>
       <c r="D1714" s="2" t="s">
         <v>3449</v>
       </c>
@@ -65511,7 +65502,7 @@
       <c r="B1715" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1715" s="5"/>
+      <c r="C1715" s="4"/>
       <c r="D1715" s="2" t="s">
         <v>3451</v>
       </c>
@@ -65541,7 +65532,7 @@
       <c r="B1716" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1716" s="5"/>
+      <c r="C1716" s="4"/>
       <c r="D1716" s="2" t="s">
         <v>3453</v>
       </c>
@@ -65571,7 +65562,7 @@
       <c r="B1717" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1717" s="5"/>
+      <c r="C1717" s="4"/>
       <c r="D1717" s="2" t="s">
         <v>3455</v>
       </c>
@@ -65601,7 +65592,7 @@
       <c r="B1718" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1718" s="5"/>
+      <c r="C1718" s="4"/>
       <c r="D1718" s="2" t="s">
         <v>3457</v>
       </c>
@@ -65631,7 +65622,7 @@
       <c r="B1719" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1719" s="5"/>
+      <c r="C1719" s="4"/>
       <c r="D1719" s="2" t="s">
         <v>3459</v>
       </c>
@@ -65661,7 +65652,7 @@
       <c r="B1720" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1720" s="5"/>
+      <c r="C1720" s="4"/>
       <c r="D1720" s="2" t="s">
         <v>3461</v>
       </c>
@@ -65691,7 +65682,7 @@
       <c r="B1721" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1721" s="5"/>
+      <c r="C1721" s="4"/>
       <c r="D1721" s="2" t="s">
         <v>3463</v>
       </c>
@@ -65721,7 +65712,7 @@
       <c r="B1722" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1722" s="5"/>
+      <c r="C1722" s="4"/>
       <c r="D1722" s="2" t="s">
         <v>3465</v>
       </c>
@@ -65751,7 +65742,7 @@
       <c r="B1723" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1723" s="5"/>
+      <c r="C1723" s="4"/>
       <c r="D1723" s="2" t="s">
         <v>3467</v>
       </c>
@@ -65781,7 +65772,7 @@
       <c r="B1724" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1724" s="5"/>
+      <c r="C1724" s="4"/>
       <c r="D1724" s="2" t="s">
         <v>3469</v>
       </c>
@@ -65811,7 +65802,7 @@
       <c r="B1725" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1725" s="5"/>
+      <c r="C1725" s="4"/>
       <c r="D1725" s="2" t="s">
         <v>3471</v>
       </c>
@@ -65841,7 +65832,7 @@
       <c r="B1726" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1726" s="5"/>
+      <c r="C1726" s="4"/>
       <c r="D1726" s="2" t="s">
         <v>3473</v>
       </c>
@@ -65871,7 +65862,7 @@
       <c r="B1727" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1727" s="5"/>
+      <c r="C1727" s="4"/>
       <c r="D1727" s="2" t="s">
         <v>3475</v>
       </c>
@@ -65901,7 +65892,7 @@
       <c r="B1728" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1728" s="5"/>
+      <c r="C1728" s="4"/>
       <c r="D1728" s="2" t="s">
         <v>3478</v>
       </c>
@@ -65931,7 +65922,7 @@
       <c r="B1729" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1729" s="5"/>
+      <c r="C1729" s="4"/>
       <c r="D1729" s="2" t="s">
         <v>3480</v>
       </c>
@@ -65961,7 +65952,7 @@
       <c r="B1730" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1730" s="5"/>
+      <c r="C1730" s="4"/>
       <c r="D1730" s="2" t="s">
         <v>3482</v>
       </c>
@@ -65991,7 +65982,7 @@
       <c r="B1731" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1731" s="5"/>
+      <c r="C1731" s="4"/>
       <c r="D1731" s="2" t="s">
         <v>3484</v>
       </c>
@@ -66021,7 +66012,7 @@
       <c r="B1732" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1732" s="5"/>
+      <c r="C1732" s="4"/>
       <c r="D1732" s="2" t="s">
         <v>3486</v>
       </c>
@@ -66051,7 +66042,7 @@
       <c r="B1733" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1733" s="5"/>
+      <c r="C1733" s="4"/>
       <c r="D1733" s="2" t="s">
         <v>3488</v>
       </c>
@@ -66081,7 +66072,7 @@
       <c r="B1734" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1734" s="5"/>
+      <c r="C1734" s="4"/>
       <c r="D1734" s="2" t="s">
         <v>3490</v>
       </c>
@@ -66111,7 +66102,7 @@
       <c r="B1735" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1735" s="5"/>
+      <c r="C1735" s="4"/>
       <c r="D1735" s="2" t="s">
         <v>3492</v>
       </c>
@@ -66141,7 +66132,7 @@
       <c r="B1736" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1736" s="5"/>
+      <c r="C1736" s="4"/>
       <c r="D1736" s="2" t="s">
         <v>3494</v>
       </c>
@@ -66171,7 +66162,7 @@
       <c r="B1737" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1737" s="5"/>
+      <c r="C1737" s="4"/>
       <c r="D1737" s="2" t="s">
         <v>3496</v>
       </c>
@@ -66201,7 +66192,7 @@
       <c r="B1738" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1738" s="5"/>
+      <c r="C1738" s="4"/>
       <c r="D1738" s="2" t="s">
         <v>3498</v>
       </c>
@@ -66231,7 +66222,7 @@
       <c r="B1739" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1739" s="5"/>
+      <c r="C1739" s="4"/>
       <c r="D1739" s="2" t="s">
         <v>3500</v>
       </c>
@@ -66261,7 +66252,7 @@
       <c r="B1740" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1740" s="5"/>
+      <c r="C1740" s="4"/>
       <c r="D1740" s="2" t="s">
         <v>3503</v>
       </c>
@@ -66291,7 +66282,7 @@
       <c r="B1741" s="2" t="s">
         <v>3427</v>
       </c>
-      <c r="C1741" s="5"/>
+      <c r="C1741" s="4"/>
       <c r="D1741" s="2" t="s">
         <v>3505</v>
       </c>

</xml_diff>